<commit_message>
made compare_timetable compatible with all data
</commit_message>
<xml_diff>
--- a/multiSchoolOutput/01_Business_School/solution_weeks_9_10.xlsx
+++ b/multiSchoolOutput/01_Business_School/solution_weeks_9_10.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0214_00_G.22</t>
+          <t>0228_07_7.01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 17:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0335_00_G.01</t>
+          <t>0450_02_2.35</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -569,7 +569,7 @@
         <v>120</v>
       </c>
       <c r="F3" t="n">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 10:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0005_02_2.01</t>
+          <t>0210_-1_B.51</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0227_00_G.05</t>
+          <t>0226_01_1.12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Friday 15:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0228_11_11.06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Monday 10:00</t>
+          <t>Wednesday 09:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -996,7 +996,7 @@
         <v>17</v>
       </c>
       <c r="F10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0005_01_1.01</t>
+          <t>0005_02_2.01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0209_01_1.21</t>
+          <t>0450_02_2.35</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1118,7 +1118,7 @@
         <v>125</v>
       </c>
       <c r="F12" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0219_00_G.02</t>
+          <t>0003_01_1.03</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0228_06_6.10</t>
+          <t>0201_04_4.14</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0335_05_5.3</t>
+          <t>0201_02_2.14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1301,7 +1301,7 @@
         <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0228_11_11.18</t>
+          <t>0228_07_7.18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1484,7 +1484,7 @@
         <v>80</v>
       </c>
       <c r="F18" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0335_00_G.09</t>
+          <t>0335_00_G.10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0226_01_1.02</t>
+          <t>0005_00_G.01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1606,7 +1606,7 @@
         <v>50</v>
       </c>
       <c r="F20" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0228_-1_LG.07</t>
+          <t>0335_04_4.3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0228_04_4.18</t>
+          <t>0008_01_1.302</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 13:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0227_03_3.14</t>
+          <t>0110_02_2.02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Friday 13:00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 15:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0113_00_G.16</t>
+          <t>0008_02_2.403</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Thursday 12:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0226_00_GF.Z16</t>
+          <t>0113_00_G.152</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Wednesday 13:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Thursday 10:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Tuesday 10:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0214_00_G.22</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2338,7 +2338,7 @@
         <v>17</v>
       </c>
       <c r="F32" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2382,12 +2382,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0113_00_G.152</t>
+          <t>0226_00_GF.Z16</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 12:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 17:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0201_07_7.14</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 09:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2521,7 +2521,7 @@
         <v>17</v>
       </c>
       <c r="F35" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 10:00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2626,12 +2626,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0113_02_2.26</t>
+          <t>0112_02_2.11</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0201_07_7.14</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2826,7 +2826,7 @@
         <v>17</v>
       </c>
       <c r="F40" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2992,12 +2992,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3009,7 +3009,7 @@
         <v>90</v>
       </c>
       <c r="F43" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0228_07_7.01</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tuesday 10:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3070,7 +3070,7 @@
         <v>17</v>
       </c>
       <c r="F44" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 10:00</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3175,12 +3175,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0113_00_G.16</t>
+          <t>0008_02_2.403</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0001_00_G.159</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3253,7 +3253,7 @@
         <v>100</v>
       </c>
       <c r="F47" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3297,12 +3297,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0201_02_2.06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3314,7 +3314,7 @@
         <v>17</v>
       </c>
       <c r="F48" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3436,7 +3436,7 @@
         <v>85</v>
       </c>
       <c r="F50" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0228_-1_LG.07</t>
+          <t>0422_J_J.05</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3663,12 +3663,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0227_01_1.06</t>
+          <t>0335_04_4.3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 12:00</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3724,12 +3724,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0229_01_1.B</t>
+          <t>0229_01_1.C</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 16:00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3968,12 +3968,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0214_00_G.26</t>
+          <t>0112_02_2.11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 16:00</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4107,7 +4107,7 @@
         <v>85</v>
       </c>
       <c r="F61" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4151,12 +4151,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0214_01_1.01</t>
+          <t>0201_01_1.01</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Thursday 12:00</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0008_02_2.418</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 17:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4290,7 +4290,7 @@
         <v>17</v>
       </c>
       <c r="F64" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -4334,12 +4334,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0228_09_9.18</t>
+          <t>0228_04_4.18</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 11:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4456,12 +4456,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0214_00_G.02</t>
+          <t>0335_03_3.3</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4578,12 +4578,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Wednesday 11:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Wednesday 13:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Wednesday 14:00</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4761,12 +4761,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>0227_01_1.02</t>
+          <t>0113_01_1.9</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4822,12 +4822,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>0210_-1_B.51</t>
+          <t>0005_02_2.01</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4883,12 +4883,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>0227_01_1.02</t>
+          <t>0311_01_1.26</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5005,12 +5005,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0228_11_11.06</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Tuesday 17:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5022,7 +5022,7 @@
         <v>17</v>
       </c>
       <c r="F76" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5127,12 +5127,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0226_01_1.02</t>
+          <t>0450_01_1.40</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5144,7 +5144,7 @@
         <v>50</v>
       </c>
       <c r="F78" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -5205,7 +5205,7 @@
         <v>85</v>
       </c>
       <c r="F79" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -5249,12 +5249,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>0228_-1_LG.09</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5266,7 +5266,7 @@
         <v>96</v>
       </c>
       <c r="F80" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5432,12 +5432,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0209_-1_B.Z28</t>
+          <t>0227_01_1.06</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5554,12 +5554,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0226_00_GF.Z16</t>
+          <t>0113_00_G.152</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Thursday 13:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5615,12 +5615,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Wednesday 11:00</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5632,7 +5632,7 @@
         <v>80</v>
       </c>
       <c r="F86" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -5676,12 +5676,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>0228_04_4.18</t>
+          <t>0110_02_2.01</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Tuesday 16:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5798,12 +5798,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>0113_02_2.65</t>
+          <t>0209_02_2.01</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5859,12 +5859,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>0228_-1_LG.09</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5876,7 +5876,7 @@
         <v>96</v>
       </c>
       <c r="F90" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 16:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5981,12 +5981,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0227_00_G.01</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Wednesday 16:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5998,7 +5998,7 @@
         <v>30</v>
       </c>
       <c r="F92" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -6042,12 +6042,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>0226_01_1.02</t>
+          <t>0450_02_2.20</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6059,7 +6059,7 @@
         <v>50</v>
       </c>
       <c r="F93" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6164,12 +6164,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0214_01_1.22</t>
+          <t>0112_04_4.11</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6225,12 +6225,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>0005_01_1.01</t>
+          <t>0210_-1_B.51</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6286,12 +6286,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>0003_01_1.02</t>
+          <t>0008_00_G.251</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6408,12 +6408,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 14:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6425,7 +6425,7 @@
         <v>30</v>
       </c>
       <c r="F99" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -6469,12 +6469,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>0227_00_G.05</t>
+          <t>0335_02_2.2</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6591,12 +6591,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>0422_J_J.05</t>
+          <t>0335_04_4.3</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 13:00</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6652,12 +6652,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6669,7 +6669,7 @@
         <v>80</v>
       </c>
       <c r="F103" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -6713,12 +6713,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>0228_09_9.18</t>
+          <t>0008_01_1.302</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 16:00</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6896,12 +6896,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0201_07_7.14</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Tuesday 17:00</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6913,7 +6913,7 @@
         <v>17</v>
       </c>
       <c r="F107" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -6957,12 +6957,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0113_00_G.03</t>
+          <t>0201_02_2.14</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6974,7 +6974,7 @@
         <v>50</v>
       </c>
       <c r="F108" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -7018,12 +7018,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0226_-1_LG.19</t>
+          <t>0113_02_2.65</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -7079,12 +7079,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0201_02_2.06</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Wednesday 09:00</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7096,7 +7096,7 @@
         <v>17</v>
       </c>
       <c r="F110" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -7140,12 +7140,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>0113_02_2.65</t>
+          <t>0226_-1_LG.19</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7262,7 +7262,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>0113_00_G.03</t>
+          <t>0005_00_G.01</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7279,7 +7279,7 @@
         <v>50</v>
       </c>
       <c r="F113" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>0228_03_3.01</t>
+          <t>0001_01_1.266</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7384,12 +7384,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>0226_-1_LG.10</t>
+          <t>0228_-1_LG.11</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7401,7 +7401,7 @@
         <v>72</v>
       </c>
       <c r="F115" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -7450,7 +7450,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Thursday 13:00</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7567,7 +7567,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>0219_00_G.01</t>
+          <t>0300_00_NG.04</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -7628,12 +7628,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>0226_-1_LG.19</t>
+          <t>0209_02_2.01</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Thursday 15:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7689,12 +7689,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Wednesday 16:00</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7706,7 +7706,7 @@
         <v>80</v>
       </c>
       <c r="F120" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Thursday 10:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7811,12 +7811,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>0335_02_2.2</t>
+          <t>0335_01_1.2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7872,12 +7872,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7889,7 +7889,7 @@
         <v>95</v>
       </c>
       <c r="F123" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -7938,7 +7938,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7994,12 +7994,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Thursday 16:00</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -8011,7 +8011,7 @@
         <v>90</v>
       </c>
       <c r="F125" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>0209_02_2.01</t>
+          <t>0113_02_2.65</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -8116,12 +8116,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>0209_02_2.01</t>
+          <t>0113_02_2.65</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -8177,12 +8177,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -8194,7 +8194,7 @@
         <v>80</v>
       </c>
       <c r="F128" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -8243,7 +8243,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8299,12 +8299,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>0209_02_2.01</t>
+          <t>0226_-1_LG.19</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Thursday 15:00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -8360,12 +8360,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>0201_04_4.14</t>
+          <t>0228_06_6.10</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8482,12 +8482,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>0008_03_3.454</t>
+          <t>0422_J_J.05</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -8543,12 +8543,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>0001_01_1.275</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8560,7 +8560,7 @@
         <v>30</v>
       </c>
       <c r="F134" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -8604,12 +8604,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>0005_01_1.01</t>
+          <t>0210_-1_B.51</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8665,12 +8665,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0113_00_G.03</t>
+          <t>0201_02_2.12</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8682,7 +8682,7 @@
         <v>50</v>
       </c>
       <c r="F136" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -8726,12 +8726,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0226_00_GF.Z16</t>
+          <t>0113_00_G.152</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8787,12 +8787,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0228_-1_LG.06</t>
+          <t>0112_-1_B.01</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8848,12 +8848,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>0335_00_G.01</t>
+          <t>0450_02_2.35</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8865,7 +8865,7 @@
         <v>120</v>
       </c>
       <c r="F139" t="n">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -8909,12 +8909,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Wednesday 09:00</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8926,7 +8926,7 @@
         <v>90</v>
       </c>
       <c r="F140" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Thursday 12:00</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -9031,12 +9031,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>0003_01_1.03</t>
+          <t>0201_02_2.05</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -9092,12 +9092,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>0335_05_5.3</t>
+          <t>0450_01_1.50</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -9109,7 +9109,7 @@
         <v>50</v>
       </c>
       <c r="F143" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -9153,12 +9153,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>0001_00_G.158</t>
+          <t>0008_00_G.267</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>0110_02_2.04</t>
+          <t>0201_03_3.01</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -9275,12 +9275,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>0335_00_G.12</t>
+          <t>0003_02_2.01</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Thursday 17:00</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -9292,7 +9292,7 @@
         <v>17</v>
       </c>
       <c r="F146" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -9336,12 +9336,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>0226_01_1.02</t>
+          <t>0450_02_2.20</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -9353,7 +9353,7 @@
         <v>50</v>
       </c>
       <c r="F147" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -9397,12 +9397,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 16:00</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -9414,7 +9414,7 @@
         <v>80</v>
       </c>
       <c r="F148" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -9458,12 +9458,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -9475,7 +9475,7 @@
         <v>80</v>
       </c>
       <c r="F149" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Tuesday 15:00</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -9702,12 +9702,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>0209_01_1.21</t>
+          <t>0450_02_2.35</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -9719,7 +9719,7 @@
         <v>125</v>
       </c>
       <c r="F153" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -9763,12 +9763,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0450_04_4.35</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 13:00</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -9824,12 +9824,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>0008_02_2.403</t>
+          <t>0113_00_G.16</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -9946,12 +9946,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>0113_00_G.152</t>
+          <t>0226_00_GF.Z16</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Wednesday 13:00</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -10007,12 +10007,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_06_6.06</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Wednesday 14:00</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -10024,7 +10024,7 @@
         <v>85</v>
       </c>
       <c r="F158" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -10068,12 +10068,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>0003_00_G.01</t>
+          <t>0210_00_GFS2</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -10129,12 +10129,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>0228_07_7.18</t>
+          <t>0113_02_2.36</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -10195,7 +10195,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Thursday 10:00</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 17:00</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -10312,12 +10312,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>0422_J_J.05</t>
+          <t>0422_J_J.03</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -10371,12 +10371,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>0201_01_1.06</t>
+          <t>0201_01_1.08</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -10388,7 +10388,7 @@
         <v>300</v>
       </c>
       <c r="F164" t="n">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -10430,12 +10430,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 16:00</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -10447,7 +10447,7 @@
         <v>90</v>
       </c>
       <c r="F165" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -10494,7 +10494,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -10548,12 +10548,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>0001_01_1.275</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -10565,7 +10565,7 @@
         <v>30</v>
       </c>
       <c r="F167" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -10607,12 +10607,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>0008_00_G.267</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Wednesday 12:00</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -10624,7 +10624,7 @@
         <v>30</v>
       </c>
       <c r="F168" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -10671,7 +10671,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -10725,12 +10725,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>0227_00_G.01</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -10742,7 +10742,7 @@
         <v>30</v>
       </c>
       <c r="F170" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -10784,12 +10784,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>0311_02_2.02</t>
+          <t>0008_03_3.454</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 09:00</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -10902,12 +10902,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>0335_01_1.3</t>
+          <t>0227_00_G.01</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 13:00</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -10961,12 +10961,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>0335_01_1.3</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Thursday 15:00</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -10978,7 +10978,7 @@
         <v>30</v>
       </c>
       <c r="F174" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -11020,12 +11020,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>0227_01_1.06</t>
+          <t>0228_-1_LG.07</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -11079,12 +11079,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>0228_-1_LG.07</t>
+          <t>0422_J_J.03</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Wednesday 15:00</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -11315,12 +11315,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>0110_02_2.02</t>
+          <t>0219_00_G.01</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -11332,7 +11332,7 @@
         <v>15</v>
       </c>
       <c r="F180" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -11374,12 +11374,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>0228_13_13.07</t>
+          <t>0219_00_G.01</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -11391,7 +11391,7 @@
         <v>15</v>
       </c>
       <c r="F181" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -11433,12 +11433,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0228_-1_LG.09</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Tuesday 11:00</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -11450,7 +11450,7 @@
         <v>85</v>
       </c>
       <c r="F182" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -11492,12 +11492,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>0214_01_1.22</t>
+          <t>0112_04_4.11</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 09:00</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -11551,12 +11551,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>0335_04_4.1</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -11568,7 +11568,7 @@
         <v>30</v>
       </c>
       <c r="F184" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -11610,12 +11610,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>0311_02_2.13</t>
+          <t>0001_00_G.159</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -11627,7 +11627,7 @@
         <v>80</v>
       </c>
       <c r="F185" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -11669,12 +11669,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>0335_00_G.01</t>
+          <t>0450_02_2.35</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Thursday 15:00</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -11686,7 +11686,7 @@
         <v>120</v>
       </c>
       <c r="F186" t="n">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -11728,12 +11728,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -11787,12 +11787,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>0227_02_2.29</t>
+          <t>0001_02_2.351</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -11804,7 +11804,7 @@
         <v>15</v>
       </c>
       <c r="F188" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -11846,12 +11846,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>0335_01_1.3</t>
+          <t>0209_02_2.37</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -11905,12 +11905,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>0228_11_11.11</t>
+          <t>0001_02_2.351</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -11922,7 +11922,7 @@
         <v>15</v>
       </c>
       <c r="F190" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -11969,7 +11969,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 11:00</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -12025,12 +12025,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>0310_00_G.06</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Wednesday 10:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -12042,7 +12042,7 @@
         <v>85</v>
       </c>
       <c r="F192" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -12091,7 +12091,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 15:00</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Thursday 16:00</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -12208,12 +12208,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Wednesday 11:00</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Wednesday 13:00</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -12330,12 +12330,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>0201_00_G.06</t>
+          <t>0201_00_G.08</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -12391,12 +12391,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Thursday 11:00</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -12450,12 +12450,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Tuesday 16:00</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -12467,7 +12467,7 @@
         <v>30</v>
       </c>
       <c r="F199" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -12511,12 +12511,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Friday 12:00</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -12528,7 +12528,7 @@
         <v>30</v>
       </c>
       <c r="F200" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -12572,12 +12572,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>0227_00_G.01</t>
+          <t>0209_02_2.37</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -12633,12 +12633,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0335_04_4.1</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Friday 14:00</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -12694,12 +12694,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -12711,7 +12711,7 @@
         <v>30</v>
       </c>
       <c r="F203" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -12755,12 +12755,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Thursday 13:00</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -12772,7 +12772,7 @@
         <v>30</v>
       </c>
       <c r="F204" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -12816,7 +12816,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>0227_00_G.01</t>
+          <t>0311_02_2.05</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -12833,7 +12833,7 @@
         <v>30</v>
       </c>
       <c r="F205" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -12877,12 +12877,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>0008_00_G.267</t>
+          <t>0450_04_4.35</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Friday 16:00</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">

</xml_diff>

<commit_message>
final results and updated penaltyTable
</commit_message>
<xml_diff>
--- a/multiSchoolOutput/01_Business_School/solution_weeks_9_10.xlsx
+++ b/multiSchoolOutput/01_Business_School/solution_weeks_9_10.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0228_07_7.01</t>
+          <t>0214_00_G.22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0450_02_2.35</t>
+          <t>0335_00_G.01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -569,7 +569,7 @@
         <v>120</v>
       </c>
       <c r="F3" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -613,12 +613,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0228_12_12.18</t>
+          <t>0228_06_6.10</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tuesday 10:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0210_-1_B.51</t>
+          <t>0005_01_1.01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -735,12 +735,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0226_01_1.12</t>
+          <t>0227_00_G.05</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Friday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -857,12 +857,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0113_00_G.152</t>
+          <t>0226_00_GF.Z16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0228_12_12.18</t>
+          <t>0201_04_4.14</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0228_11_11.06</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -996,7 +996,7 @@
         <v>17</v>
       </c>
       <c r="F10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0450_02_2.35</t>
+          <t>0209_01_1.21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1118,7 +1118,7 @@
         <v>125</v>
       </c>
       <c r="F12" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0003_01_1.03</t>
+          <t>0113_02_2.36</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Monday 10:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0201_02_2.14</t>
+          <t>0226_01_1.02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1301,7 +1301,7 @@
         <v>50</v>
       </c>
       <c r="F15" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0228_07_7.18</t>
+          <t>0001_01_1.266</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0228_11_11.11</t>
+          <t>0113_00_G.10</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1484,7 +1484,7 @@
         <v>80</v>
       </c>
       <c r="F18" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0335_00_G.10</t>
+          <t>0335_00_G.09</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0005_00_G.01</t>
+          <t>0113_00_G.03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1606,7 +1606,7 @@
         <v>50</v>
       </c>
       <c r="F20" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0335_04_4.3</t>
+          <t>0227_01_1.06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tuesday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Friday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0110_02_2.02</t>
+          <t>0227_02_2.14</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Friday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tuesday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0008_02_2.403</t>
+          <t>0113_00_G.16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thursday 12:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wednesday 13:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0005_02_2.01</t>
+          <t>0210_-1_B.51</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thursday 10:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2199,12 +2199,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0228_06_6.10</t>
+          <t>0201_04_4.14</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tuesday 10:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0214_00_G.22</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Tuesday 10:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2338,7 +2338,7 @@
         <v>17</v>
       </c>
       <c r="F32" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Thursday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0201_07_7.14</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2521,7 +2521,7 @@
         <v>17</v>
       </c>
       <c r="F35" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2565,12 +2565,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0210_-1_B.51</t>
+          <t>0005_01_1.01</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Tuesday 10:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2626,12 +2626,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0112_02_2.11</t>
+          <t>0214_01_1.22</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0201_02_2.07</t>
+          <t>0210_00_GFS2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0201_07_7.14</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2826,7 +2826,7 @@
         <v>17</v>
       </c>
       <c r="F40" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2931,12 +2931,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0226_00_GF.Z16</t>
+          <t>0113_00_G.152</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2992,12 +2992,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3009,7 +3009,7 @@
         <v>90</v>
       </c>
       <c r="F43" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0228_07_7.01</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3070,7 +3070,7 @@
         <v>17</v>
       </c>
       <c r="F44" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0201_04_4.14</t>
+          <t>0228_12_12.18</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tuesday 10:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3175,12 +3175,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0008_02_2.403</t>
+          <t>0113_00_G.16</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0001_00_G.159</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3253,7 +3253,7 @@
         <v>100</v>
       </c>
       <c r="F47" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3297,12 +3297,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0201_02_2.06</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3314,7 +3314,7 @@
         <v>17</v>
       </c>
       <c r="F48" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3436,7 +3436,7 @@
         <v>85</v>
       </c>
       <c r="F50" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Thursday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Thursday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3968,12 +3968,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0112_02_2.11</t>
+          <t>0113_01M_01M.27</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4029,12 +4029,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0228_04_4.18</t>
+          <t>0228_09_9.18</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Monday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4090,12 +4090,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4107,7 +4107,7 @@
         <v>85</v>
       </c>
       <c r="F61" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4151,12 +4151,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0201_01_1.01</t>
+          <t>0113_01_1.42</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4212,12 +4212,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0113_00_G.16</t>
+          <t>0008_02_2.403</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Thursday 12:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0008_02_2.418</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Tuesday 13:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4290,7 +4290,7 @@
         <v>17</v>
       </c>
       <c r="F64" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -4334,12 +4334,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0228_04_4.18</t>
+          <t>0335_02_2.1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Monday 11:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4456,12 +4456,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0335_03_3.3</t>
+          <t>0227_01_1.02</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4578,12 +4578,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Wednesday 11:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Wednesday 13:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4700,12 +4700,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0228_04_4.18</t>
+          <t>0113_01M_01M.467</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Wednesday 14:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4883,12 +4883,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>0311_01_1.26</t>
+          <t>0113_01M_01M.469</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5005,12 +5005,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0228_11_11.06</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5022,7 +5022,7 @@
         <v>17</v>
       </c>
       <c r="F76" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5066,12 +5066,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>0335_02_2.3</t>
+          <t>0214_00_G.02</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5127,12 +5127,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0450_01_1.40</t>
+          <t>0226_01_1.02</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5144,7 +5144,7 @@
         <v>50</v>
       </c>
       <c r="F78" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -5188,12 +5188,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5205,7 +5205,7 @@
         <v>85</v>
       </c>
       <c r="F79" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -5249,12 +5249,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0228_-1_LG.09</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5266,7 +5266,7 @@
         <v>96</v>
       </c>
       <c r="F80" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Tuesday 13:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5371,12 +5371,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>0209_02_2.01</t>
+          <t>0113_02_2.65</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5432,12 +5432,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0227_01_1.06</t>
+          <t>0209_-1_B.Z28</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Tuesday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Thursday 13:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5615,12 +5615,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Wednesday 11:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5632,7 +5632,7 @@
         <v>80</v>
       </c>
       <c r="F86" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -5676,12 +5676,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>0110_02_2.01</t>
+          <t>0008_01_1.302</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Tuesday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Monday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5859,12 +5859,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0228_-1_LG.09</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5876,7 +5876,7 @@
         <v>96</v>
       </c>
       <c r="F90" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Monday 16:00</t>
+          <t>Tuesday 15:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5981,12 +5981,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_01_1.275</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Wednesday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5998,7 +5998,7 @@
         <v>30</v>
       </c>
       <c r="F92" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -6042,12 +6042,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>0450_02_2.20</t>
+          <t>0113_00_G.03</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6059,7 +6059,7 @@
         <v>50</v>
       </c>
       <c r="F93" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6164,12 +6164,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0112_04_4.11</t>
+          <t>0113_02_2.27</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6286,12 +6286,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>0008_00_G.251</t>
+          <t>0450_03_3.52</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6408,12 +6408,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0335_04_4.1</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Wednesday 14:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6425,7 +6425,7 @@
         <v>30</v>
       </c>
       <c r="F99" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6591,12 +6591,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>0335_04_4.3</t>
+          <t>0311_02_2.02</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Thursday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6652,12 +6652,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6669,7 +6669,7 @@
         <v>80</v>
       </c>
       <c r="F103" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -6713,12 +6713,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>0008_01_1.302</t>
+          <t>0335_05_5.1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Thursday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6774,12 +6774,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>0008_02_2.403</t>
+          <t>0113_00_G.16</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6835,12 +6835,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>0227_00_G.05</t>
+          <t>0335_02_2.2</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6896,12 +6896,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>0201_07_7.14</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Tuesday 17:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6913,7 +6913,7 @@
         <v>17</v>
       </c>
       <c r="F107" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -6957,12 +6957,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0201_02_2.14</t>
+          <t>0335_05_5.3</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6974,7 +6974,7 @@
         <v>50</v>
       </c>
       <c r="F108" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -7018,12 +7018,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0113_02_2.65</t>
+          <t>0209_02_2.01</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -7079,12 +7079,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>0201_02_2.06</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7096,7 +7096,7 @@
         <v>17</v>
       </c>
       <c r="F110" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -7145,7 +7145,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Monday 15:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7262,12 +7262,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>0005_00_G.01</t>
+          <t>0113_00_G.03</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7279,7 +7279,7 @@
         <v>50</v>
       </c>
       <c r="F113" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>0001_01_1.266</t>
+          <t>0008_00_G.251</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7384,12 +7384,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>0228_-1_LG.11</t>
+          <t>0226_-1_LG.10</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7401,7 +7401,7 @@
         <v>72</v>
       </c>
       <c r="F115" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -7445,12 +7445,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>0422_J_J.05</t>
+          <t>0008_03_3.454</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Thursday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7567,12 +7567,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>0300_00_NG.04</t>
+          <t>0001_02_2.351</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7628,12 +7628,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>0209_02_2.01</t>
+          <t>0113_02_2.65</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Thursday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7689,12 +7689,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Wednesday 16:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7706,7 +7706,7 @@
         <v>80</v>
       </c>
       <c r="F120" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Monday 15:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7811,12 +7811,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>0335_01_1.2</t>
+          <t>0335_02_2.2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7872,12 +7872,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0201_01_1.02</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7889,7 +7889,7 @@
         <v>95</v>
       </c>
       <c r="F123" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -7933,12 +7933,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>0113_00_G.16</t>
+          <t>0008_02_2.403</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7994,12 +7994,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Thursday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -8011,7 +8011,7 @@
         <v>90</v>
       </c>
       <c r="F125" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>0113_02_2.65</t>
+          <t>0209_02_2.01</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -8116,12 +8116,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>0113_02_2.65</t>
+          <t>0226_-1_LG.19</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Monday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -8177,12 +8177,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -8194,7 +8194,7 @@
         <v>80</v>
       </c>
       <c r="F128" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -8243,7 +8243,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Thursday 15:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -8360,12 +8360,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>0228_06_6.10</t>
+          <t>0228_12_12.18</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Monday 10:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -8543,12 +8543,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0209_02_2.37</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8560,7 +8560,7 @@
         <v>30</v>
       </c>
       <c r="F134" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8665,12 +8665,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0201_02_2.12</t>
+          <t>0335_05_5.3</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8682,7 +8682,7 @@
         <v>50</v>
       </c>
       <c r="F136" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -8726,12 +8726,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0113_00_G.152</t>
+          <t>0226_00_GF.Z16</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Tuesday 13:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8787,12 +8787,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0112_-1_B.01</t>
+          <t>0113_00M_00M.05</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8848,12 +8848,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>0450_02_2.35</t>
+          <t>0335_00_G.01</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8865,7 +8865,7 @@
         <v>120</v>
       </c>
       <c r="F139" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -8909,12 +8909,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Wednesday 09:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8926,7 +8926,7 @@
         <v>90</v>
       </c>
       <c r="F140" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -8970,12 +8970,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>0113_00M_00M.05</t>
+          <t>0228_-1_LG.06</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Thursday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -9031,12 +9031,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>0201_02_2.05</t>
+          <t>0228_03_3.01</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -9092,12 +9092,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>0450_01_1.50</t>
+          <t>0335_05_5.3</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -9109,7 +9109,7 @@
         <v>50</v>
       </c>
       <c r="F143" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -9153,12 +9153,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>0008_00_G.267</t>
+          <t>0450_04_4.35</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -9214,12 +9214,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>0201_03_3.01</t>
+          <t>0110_02_2.04</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Monday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -9275,12 +9275,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>0003_02_2.01</t>
+          <t>0335_00_G.12</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Thursday 17:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -9292,7 +9292,7 @@
         <v>17</v>
       </c>
       <c r="F146" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -9336,12 +9336,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>0450_02_2.20</t>
+          <t>0113_00_G.03</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 14:00</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -9353,7 +9353,7 @@
         <v>50</v>
       </c>
       <c r="F147" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -9397,12 +9397,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Tuesday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -9414,7 +9414,7 @@
         <v>80</v>
       </c>
       <c r="F148" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -9458,12 +9458,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Tuesday 13:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -9475,7 +9475,7 @@
         <v>80</v>
       </c>
       <c r="F149" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -9585,7 +9585,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Tuesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -9702,12 +9702,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>0450_02_2.35</t>
+          <t>0209_01_1.21</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -9719,7 +9719,7 @@
         <v>125</v>
       </c>
       <c r="F153" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -9763,12 +9763,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0008_00_G.267</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Friday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -9824,12 +9824,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>0113_00_G.16</t>
+          <t>0008_02_2.403</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Wednesday 13:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -10007,12 +10007,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>0201_06_6.06</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Wednesday 14:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -10024,7 +10024,7 @@
         <v>85</v>
       </c>
       <c r="F158" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -10068,12 +10068,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>0210_00_GFS2</t>
+          <t>0003_00_G.01</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -10129,12 +10129,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>0113_02_2.36</t>
+          <t>0219_00_G.02</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -10195,7 +10195,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Thursday 10:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -10251,12 +10251,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>0103_01_1.B09</t>
+          <t>0001_02_2.349</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Wednesday 17:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -10317,7 +10317,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -10371,12 +10371,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>0201_01_1.08</t>
+          <t>0201_01_1.06</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -10388,7 +10388,7 @@
         <v>300</v>
       </c>
       <c r="F164" t="n">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -10430,12 +10430,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Wednesday 16:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -10447,7 +10447,7 @@
         <v>90</v>
       </c>
       <c r="F165" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -10494,7 +10494,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Monday 09:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -10548,12 +10548,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0209_02_2.37</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -10565,7 +10565,7 @@
         <v>30</v>
       </c>
       <c r="F167" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -10607,12 +10607,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0008_00_G.267</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Wednesday 12:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -10624,7 +10624,7 @@
         <v>30</v>
       </c>
       <c r="F168" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -10671,7 +10671,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -10725,12 +10725,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_01_1.275</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Monday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -10742,7 +10742,7 @@
         <v>30</v>
       </c>
       <c r="F170" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -10784,12 +10784,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>0008_03_3.454</t>
+          <t>0422_J_J.05</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -10843,12 +10843,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>0227_00_G.05</t>
+          <t>0335_01_1.2</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Friday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -10902,12 +10902,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>0227_00_G.01</t>
+          <t>0001_00_G.158</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Friday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -10961,12 +10961,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_00_G.158</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Thursday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -10978,7 +10978,7 @@
         <v>30</v>
       </c>
       <c r="F174" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -11025,7 +11025,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -11084,7 +11084,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -11197,12 +11197,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>0228_-1_LG.06</t>
+          <t>0112_-1_B.01</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Monday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -11256,12 +11256,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0227_00_G.01</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Wednesday 15:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -11315,12 +11315,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>0219_00_G.01</t>
+          <t>0228_13_13.07</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -11332,7 +11332,7 @@
         <v>15</v>
       </c>
       <c r="F180" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -11374,12 +11374,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>0219_00_G.01</t>
+          <t>0113_00_G.12</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -11391,7 +11391,7 @@
         <v>15</v>
       </c>
       <c r="F181" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -11433,12 +11433,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>0228_-1_LG.09</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Tuesday 11:00</t>
+          <t>Monday 17:00</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -11450,7 +11450,7 @@
         <v>85</v>
       </c>
       <c r="F182" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -11492,12 +11492,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>0112_04_4.11</t>
+          <t>0113_02_2.26</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Thursday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -11551,12 +11551,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0335_01_1.3</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Tuesday 14:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -11568,7 +11568,7 @@
         <v>30</v>
       </c>
       <c r="F184" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -11610,12 +11610,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>0001_00_G.159</t>
+          <t>0311_02_2.13</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Monday 12:00</t>
+          <t>Monday 13:00</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -11627,7 +11627,7 @@
         <v>80</v>
       </c>
       <c r="F185" t="n">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -11669,12 +11669,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>0450_02_2.35</t>
+          <t>0335_00_G.01</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Thursday 15:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -11686,7 +11686,7 @@
         <v>120</v>
       </c>
       <c r="F186" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -11733,7 +11733,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -11787,7 +11787,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>0001_02_2.351</t>
+          <t>0008_-1_B.154</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -11804,7 +11804,7 @@
         <v>15</v>
       </c>
       <c r="F188" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -11846,12 +11846,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0001_01_1.275</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -11905,12 +11905,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>0001_02_2.351</t>
+          <t>0008_-1_B.153</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Tuesday 09:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -11922,7 +11922,7 @@
         <v>15</v>
       </c>
       <c r="F190" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -11969,7 +11969,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Friday 11:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -12025,12 +12025,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>0201_01_1.02</t>
+          <t>0310_00_G.06</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Wednesday 09:00</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -12042,7 +12042,7 @@
         <v>85</v>
       </c>
       <c r="F192" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -12086,12 +12086,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>0201_00_G.08</t>
+          <t>0201_00_G.06</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Tuesday 15:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -12147,12 +12147,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Thursday 16:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -12208,12 +12208,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>0227_00_G.04</t>
+          <t>0310_00_G.Z02</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Wednesday 11:00</t>
+          <t>Monday 10:00</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Wednesday 13:00</t>
+          <t>Monday 09:00</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Monday 14:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -12391,12 +12391,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>0310_00_G.Z02</t>
+          <t>0227_00_G.04</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Thursday 11:00</t>
+          <t>Monday 12:00</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -12450,12 +12450,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0227_00_G.01</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Tuesday 16:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -12467,7 +12467,7 @@
         <v>30</v>
       </c>
       <c r="F199" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -12511,12 +12511,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_00_G.158</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Friday 12:00</t>
+          <t>Tuesday 09:00</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -12528,7 +12528,7 @@
         <v>30</v>
       </c>
       <c r="F200" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -12572,12 +12572,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>0209_02_2.37</t>
+          <t>0001_01_1.275</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -12633,12 +12633,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>0335_04_4.1</t>
+          <t>0227_00_G.01</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Friday 14:00</t>
+          <t>Tuesday 12:00</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -12694,12 +12694,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_00_G.158</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -12711,7 +12711,7 @@
         <v>30</v>
       </c>
       <c r="F203" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -12755,12 +12755,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_01_1.275</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Thursday 13:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -12772,7 +12772,7 @@
         <v>30</v>
       </c>
       <c r="F204" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -12816,12 +12816,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>0311_02_2.05</t>
+          <t>0001_00_G.158</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Tuesday 12:00</t>
+          <t>Tuesday 14:00</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -12833,7 +12833,7 @@
         <v>30</v>
       </c>
       <c r="F205" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -12877,12 +12877,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>0450_04_4.35</t>
+          <t>0008_00_G.267</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Friday 16:00</t>
+          <t>Monday 15:00</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">

</xml_diff>